<commit_message>
Updated Procedure Category related CS
</commit_message>
<xml_diff>
--- a/314e-ig/output/CodeSystem-procedure-category-314e.xlsx
+++ b/314e-ig/output/CodeSystem-procedure-category-314e.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="175">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-05-16T10:04:42+05:30</t>
+    <t>2026-05-16T10:41:11+05:30</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -148,6 +148,9 @@
     <t>Laboratory Medicine (In-Vitro)</t>
   </si>
   <si>
+    <t>Laboratory diagnostic services</t>
+  </si>
+  <si>
     <t>2</t>
   </si>
   <si>
@@ -157,70 +160,106 @@
     <t>Hematology &amp; Chemistry</t>
   </si>
   <si>
+    <t>Blood counts, routine panels</t>
+  </si>
+  <si>
     <t>PATH</t>
   </si>
   <si>
     <t>Pathology &amp; Cytology</t>
   </si>
   <si>
+    <t>Biopsies, cell blocks, smears</t>
+  </si>
+  <si>
     <t>MICV</t>
   </si>
   <si>
     <t>Microbiology &amp; Virology</t>
   </si>
   <si>
+    <t>Cultures, PCR tests, stains</t>
+  </si>
+  <si>
     <t>BBTM</t>
   </si>
   <si>
     <t>Transfusion Medicine / Blood Bank</t>
   </si>
   <si>
+    <t>Cross-matches, antibody screens</t>
+  </si>
+  <si>
     <t>GEND</t>
   </si>
   <si>
     <t>Molecular Diagnostics &amp; Genetics</t>
   </si>
   <si>
+    <t>Gene sequencing, karyotyping</t>
+  </si>
+  <si>
     <t>IMG</t>
   </si>
   <si>
     <t>Diagnostic Imaging (Anatomical)</t>
   </si>
   <si>
+    <t>Anatomical imaging procedures</t>
+  </si>
+  <si>
     <t>RRXG</t>
   </si>
   <si>
     <t>Routine Radiology</t>
   </si>
   <si>
+    <t>Plain X-Rays, Mammography</t>
+  </si>
+  <si>
     <t>ACSI</t>
   </si>
   <si>
     <t>Advanced Cross-Sectional</t>
   </si>
   <si>
+    <t>CT Scans, MRIs</t>
+  </si>
+  <si>
     <t>CATH</t>
   </si>
   <si>
     <t>Interventional Radiology &amp; Cath Lab Imaging</t>
   </si>
   <si>
+    <t>Angiography, Fluoroscopy</t>
+  </si>
+  <si>
     <t>NUCM</t>
   </si>
   <si>
     <t>Nuclear Medicine</t>
   </si>
   <si>
+    <t>PET Scans, SPECT Scans, Bone Scintigraphy</t>
+  </si>
+  <si>
     <t>MEDP</t>
   </si>
   <si>
     <t>Medical Photography</t>
   </si>
   <si>
+    <t>Dermatology, Ophthalmology retinal photos</t>
+  </si>
+  <si>
     <t>FNP</t>
   </si>
   <si>
-    <t>Functional &amp; Physiological Studies</t>
+    <t>Functional &amp; Physiological Studies (Non-Invasive)</t>
+  </si>
+  <si>
+    <t>Functional and physiological diagnostic procedures</t>
   </si>
   <si>
     <t>CARD</t>
@@ -229,184 +268,277 @@
     <t>Cardiology</t>
   </si>
   <si>
+    <t>EKGs, Holter monitors, Stress tests</t>
+  </si>
+  <si>
     <t>NEUS</t>
   </si>
   <si>
     <t>Neurology &amp; Sleep</t>
   </si>
   <si>
+    <t>EEGs, EMGs, Polysomnography</t>
+  </si>
+  <si>
     <t>PULM</t>
   </si>
   <si>
     <t>Pulmonary</t>
   </si>
   <si>
+    <t>PFTs, Spirometry, Blood Gas tracings</t>
+  </si>
+  <si>
     <t>AUDV</t>
   </si>
   <si>
     <t>Audiology &amp; Vestibular</t>
   </si>
   <si>
+    <t>Audiograms, Tympanometry, VNG balance tests</t>
+  </si>
+  <si>
     <t>GIFN</t>
   </si>
   <si>
     <t>Gastroenterology Functional</t>
   </si>
   <si>
+    <t>Manometry, 24-hr pH monitoring</t>
+  </si>
+  <si>
     <t>SUR</t>
   </si>
   <si>
     <t>Invasive &amp; Surgical Procedures</t>
   </si>
   <si>
+    <t>Invasive and surgical clinical procedures</t>
+  </si>
+  <si>
     <t>ORSU</t>
   </si>
   <si>
     <t>Operative &amp; Major Surgical Procedures</t>
   </si>
   <si>
+    <t>OR surgeries, day surgeries</t>
+  </si>
+  <si>
     <t>ENDO</t>
   </si>
   <si>
     <t>Endoscopic Procedures</t>
   </si>
   <si>
+    <t>GI scopes, Bronchoscopy, Cystoscopy</t>
+  </si>
+  <si>
     <t>MSUR</t>
   </si>
   <si>
     <t>Bedside &amp; Minor Invasive Procedures</t>
   </si>
   <si>
+    <t>Lumbar punctures, Paracentesis</t>
+  </si>
+  <si>
     <t>TIN</t>
   </si>
   <si>
     <t>Therapeutics &amp; Infusion Services</t>
   </si>
   <si>
+    <t>Therapeutic and infusion-based treatment services</t>
+  </si>
+  <si>
     <t>IONC</t>
   </si>
   <si>
     <t>Infusion Oncology</t>
   </si>
   <si>
+    <t>Chemotherapy, Immunotherapy biologics</t>
+  </si>
+  <si>
     <t>RONC</t>
   </si>
   <si>
     <t>Radiation Oncology</t>
   </si>
   <si>
+    <t>External beam radiation, Brachytherapy</t>
+  </si>
+  <si>
     <t>BLDT</t>
   </si>
   <si>
     <t>Renal &amp; Blood Therapies</t>
   </si>
   <si>
+    <t>Hemodialysis, Peritoneal dialysis, Apheresis</t>
+  </si>
+  <si>
     <t>INFU</t>
   </si>
   <si>
     <t>Specialty Infusions</t>
   </si>
   <si>
+    <t>IV Antibiotics, Iron infusions, Pain pumps</t>
+  </si>
+  <si>
     <t>MEDA</t>
   </si>
   <si>
     <t>Bedside &amp; General Medication Administration</t>
   </si>
   <si>
+    <t>General medication administration activities</t>
+  </si>
+  <si>
     <t>RHB</t>
   </si>
   <si>
     <t>Rehabilitative, Supportive &amp; Physical Medicine</t>
   </si>
   <si>
+    <t>Rehabilitative and supportive therapeutic services</t>
+  </si>
+  <si>
     <t>PHYT</t>
   </si>
   <si>
     <t>Physical Therapy</t>
   </si>
   <si>
+    <t>Gross motor, mobility, wound care</t>
+  </si>
+  <si>
     <t>OCCT</t>
   </si>
   <si>
     <t>Occupational Therapy</t>
   </si>
   <si>
+    <t>Fine motor, cognitive/ADL adaptations</t>
+  </si>
+  <si>
     <t>SPLP</t>
   </si>
   <si>
     <t>Speech-Language Pathology</t>
   </si>
   <si>
+    <t>Swallowing studies, cognitive speech</t>
+  </si>
+  <si>
     <t>RSPT</t>
   </si>
   <si>
     <t>Respiratory Therapy</t>
   </si>
   <si>
+    <t>Ventilator weaning, chest physiotherapy</t>
+  </si>
+  <si>
     <t>PALC</t>
   </si>
   <si>
     <t>Palliative &amp; Comfort Care Regimens</t>
   </si>
   <si>
+    <t>Symptom optimization, end-of-life care</t>
+  </si>
+  <si>
     <t>CBE</t>
   </si>
   <si>
     <t>Cognitive, Behavioral &amp; Education Services</t>
   </si>
   <si>
+    <t>Cognitive, behavioral, counseling, and educational services</t>
+  </si>
+  <si>
     <t>WELL</t>
   </si>
   <si>
     <t>Preventive &amp; Wellness Education</t>
   </si>
   <si>
+    <t>Diet tracking, smoking cessation, lactation support</t>
+  </si>
+  <si>
     <t>PSYC</t>
   </si>
   <si>
     <t>Psychological &amp; Mental Health Counseling</t>
   </si>
   <si>
+    <t>Psychotherapy, grief counseling, CBT</t>
+  </si>
+  <si>
     <t>GENC</t>
   </si>
   <si>
     <t>Genetic &amp; Familial Counseling</t>
   </si>
   <si>
+    <t>Pre-implantation counseling, oncology risk mapping</t>
+  </si>
+  <si>
     <t>MEDC</t>
   </si>
   <si>
     <t>Medication and Device Compliance Education</t>
   </si>
   <si>
+    <t>Inhaler mechanics training, anticoagulant compliance</t>
+  </si>
+  <si>
     <t>CNS</t>
   </si>
   <si>
     <t>Clinical Consultations &amp; Care Coordination</t>
   </si>
   <si>
+    <t>Consultation, coordination, referral, and transitional care services</t>
+  </si>
+  <si>
     <t>SPEC</t>
   </si>
   <si>
     <t>Specialist Consultations &amp; Referrals</t>
   </si>
   <si>
+    <t>Referral and specialist consultation workflows</t>
+  </si>
+  <si>
     <t>NURS</t>
   </si>
   <si>
     <t>Nursing &amp; Bedside Care Orders</t>
   </si>
   <si>
+    <t>Non-surgical clinical tasks executed by nursing staff</t>
+  </si>
+  <si>
     <t>SDOH</t>
   </si>
   <si>
     <t>Social &amp; Community Care Services</t>
   </si>
   <si>
+    <t>SDOH referrals including housing and food security</t>
+  </si>
+  <si>
     <t>DIST</t>
   </si>
   <si>
     <t>Discharge &amp; Transitional Care Management</t>
+  </si>
+  <si>
+    <t>Discharge planning and transitional care coordination</t>
   </si>
 </sst>
 </file>
@@ -743,523 +875,611 @@
       <c r="C2" t="s" s="2">
         <v>43</v>
       </c>
-      <c r="D2" s="2"/>
+      <c r="D2" t="s" s="2">
+        <v>44</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>46</v>
-      </c>
-      <c r="D3" s="2"/>
+        <v>47</v>
+      </c>
+      <c r="D3" t="s" s="2">
+        <v>48</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C4" t="s" s="2">
-        <v>48</v>
-      </c>
-      <c r="D4" s="2"/>
+        <v>50</v>
+      </c>
+      <c r="D4" t="s" s="2">
+        <v>51</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B5" t="s" s="2">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C5" t="s" s="2">
-        <v>50</v>
-      </c>
-      <c r="D5" s="2"/>
+        <v>53</v>
+      </c>
+      <c r="D5" t="s" s="2">
+        <v>54</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B6" t="s" s="2">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C6" t="s" s="2">
-        <v>52</v>
-      </c>
-      <c r="D6" s="2"/>
+        <v>56</v>
+      </c>
+      <c r="D6" t="s" s="2">
+        <v>57</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B7" t="s" s="2">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="C7" t="s" s="2">
-        <v>54</v>
-      </c>
-      <c r="D7" s="2"/>
+        <v>59</v>
+      </c>
+      <c r="D7" t="s" s="2">
+        <v>60</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
         <v>41</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C8" t="s" s="2">
-        <v>56</v>
-      </c>
-      <c r="D8" s="2"/>
+        <v>62</v>
+      </c>
+      <c r="D8" t="s" s="2">
+        <v>63</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="C9" t="s" s="2">
-        <v>58</v>
-      </c>
-      <c r="D9" s="2"/>
+        <v>65</v>
+      </c>
+      <c r="D9" t="s" s="2">
+        <v>66</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B10" t="s" s="2">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="C10" t="s" s="2">
-        <v>60</v>
-      </c>
-      <c r="D10" s="2"/>
+        <v>68</v>
+      </c>
+      <c r="D10" t="s" s="2">
+        <v>69</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="C11" t="s" s="2">
-        <v>62</v>
-      </c>
-      <c r="D11" s="2"/>
+        <v>71</v>
+      </c>
+      <c r="D11" t="s" s="2">
+        <v>72</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="C12" t="s" s="2">
-        <v>64</v>
-      </c>
-      <c r="D12" s="2"/>
+        <v>74</v>
+      </c>
+      <c r="D12" t="s" s="2">
+        <v>75</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="C13" t="s" s="2">
-        <v>66</v>
-      </c>
-      <c r="D13" s="2"/>
+        <v>77</v>
+      </c>
+      <c r="D13" t="s" s="2">
+        <v>78</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
         <v>41</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="C14" t="s" s="2">
-        <v>68</v>
-      </c>
-      <c r="D14" s="2"/>
+        <v>80</v>
+      </c>
+      <c r="D14" t="s" s="2">
+        <v>81</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="C15" t="s" s="2">
-        <v>70</v>
-      </c>
-      <c r="D15" s="2"/>
+        <v>83</v>
+      </c>
+      <c r="D15" t="s" s="2">
+        <v>84</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="C16" t="s" s="2">
-        <v>72</v>
-      </c>
-      <c r="D16" s="2"/>
+        <v>86</v>
+      </c>
+      <c r="D16" t="s" s="2">
+        <v>87</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="C17" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="D17" s="2"/>
+        <v>89</v>
+      </c>
+      <c r="D17" t="s" s="2">
+        <v>90</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="C18" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="D18" s="2"/>
+        <v>92</v>
+      </c>
+      <c r="D18" t="s" s="2">
+        <v>93</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>77</v>
+        <v>94</v>
       </c>
       <c r="C19" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="D19" s="2"/>
+        <v>95</v>
+      </c>
+      <c r="D19" t="s" s="2">
+        <v>96</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
         <v>41</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>79</v>
+        <v>97</v>
       </c>
       <c r="C20" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="D20" s="2"/>
+        <v>98</v>
+      </c>
+      <c r="D20" t="s" s="2">
+        <v>99</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>81</v>
+        <v>100</v>
       </c>
       <c r="C21" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="D21" s="2"/>
+        <v>101</v>
+      </c>
+      <c r="D21" t="s" s="2">
+        <v>102</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>83</v>
+        <v>103</v>
       </c>
       <c r="C22" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="D22" s="2"/>
+        <v>104</v>
+      </c>
+      <c r="D22" t="s" s="2">
+        <v>105</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>85</v>
+        <v>106</v>
       </c>
       <c r="C23" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="D23" s="2"/>
+        <v>107</v>
+      </c>
+      <c r="D23" t="s" s="2">
+        <v>108</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
         <v>41</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>87</v>
+        <v>109</v>
       </c>
       <c r="C24" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="D24" s="2"/>
+        <v>110</v>
+      </c>
+      <c r="D24" t="s" s="2">
+        <v>111</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>89</v>
+        <v>112</v>
       </c>
       <c r="C25" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="D25" s="2"/>
+        <v>113</v>
+      </c>
+      <c r="D25" t="s" s="2">
+        <v>114</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>91</v>
+        <v>115</v>
       </c>
       <c r="C26" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="D26" s="2"/>
+        <v>116</v>
+      </c>
+      <c r="D26" t="s" s="2">
+        <v>117</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>93</v>
+        <v>118</v>
       </c>
       <c r="C27" t="s" s="2">
-        <v>94</v>
-      </c>
-      <c r="D27" s="2"/>
+        <v>119</v>
+      </c>
+      <c r="D27" t="s" s="2">
+        <v>120</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>95</v>
+        <v>121</v>
       </c>
       <c r="C28" t="s" s="2">
-        <v>96</v>
-      </c>
-      <c r="D28" s="2"/>
+        <v>122</v>
+      </c>
+      <c r="D28" t="s" s="2">
+        <v>123</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>97</v>
+        <v>124</v>
       </c>
       <c r="C29" t="s" s="2">
-        <v>98</v>
-      </c>
-      <c r="D29" s="2"/>
+        <v>125</v>
+      </c>
+      <c r="D29" t="s" s="2">
+        <v>126</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
         <v>41</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>99</v>
+        <v>127</v>
       </c>
       <c r="C30" t="s" s="2">
-        <v>100</v>
-      </c>
-      <c r="D30" s="2"/>
+        <v>128</v>
+      </c>
+      <c r="D30" t="s" s="2">
+        <v>129</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>101</v>
+        <v>130</v>
       </c>
       <c r="C31" t="s" s="2">
-        <v>102</v>
-      </c>
-      <c r="D31" s="2"/>
+        <v>131</v>
+      </c>
+      <c r="D31" t="s" s="2">
+        <v>132</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>103</v>
+        <v>133</v>
       </c>
       <c r="C32" t="s" s="2">
-        <v>104</v>
-      </c>
-      <c r="D32" s="2"/>
+        <v>134</v>
+      </c>
+      <c r="D32" t="s" s="2">
+        <v>135</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>105</v>
+        <v>136</v>
       </c>
       <c r="C33" t="s" s="2">
-        <v>106</v>
-      </c>
-      <c r="D33" s="2"/>
+        <v>137</v>
+      </c>
+      <c r="D33" t="s" s="2">
+        <v>138</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>107</v>
+        <v>139</v>
       </c>
       <c r="C34" t="s" s="2">
-        <v>108</v>
-      </c>
-      <c r="D34" s="2"/>
+        <v>140</v>
+      </c>
+      <c r="D34" t="s" s="2">
+        <v>141</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>109</v>
+        <v>142</v>
       </c>
       <c r="C35" t="s" s="2">
-        <v>110</v>
-      </c>
-      <c r="D35" s="2"/>
+        <v>143</v>
+      </c>
+      <c r="D35" t="s" s="2">
+        <v>144</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
         <v>41</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>111</v>
+        <v>145</v>
       </c>
       <c r="C36" t="s" s="2">
-        <v>112</v>
-      </c>
-      <c r="D36" s="2"/>
+        <v>146</v>
+      </c>
+      <c r="D36" t="s" s="2">
+        <v>147</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>113</v>
+        <v>148</v>
       </c>
       <c r="C37" t="s" s="2">
-        <v>114</v>
-      </c>
-      <c r="D37" s="2"/>
+        <v>149</v>
+      </c>
+      <c r="D37" t="s" s="2">
+        <v>150</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>115</v>
+        <v>151</v>
       </c>
       <c r="C38" t="s" s="2">
-        <v>116</v>
-      </c>
-      <c r="D38" s="2"/>
+        <v>152</v>
+      </c>
+      <c r="D38" t="s" s="2">
+        <v>153</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>117</v>
+        <v>154</v>
       </c>
       <c r="C39" t="s" s="2">
-        <v>118</v>
-      </c>
-      <c r="D39" s="2"/>
+        <v>155</v>
+      </c>
+      <c r="D39" t="s" s="2">
+        <v>156</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>119</v>
+        <v>157</v>
       </c>
       <c r="C40" t="s" s="2">
-        <v>120</v>
-      </c>
-      <c r="D40" s="2"/>
+        <v>158</v>
+      </c>
+      <c r="D40" t="s" s="2">
+        <v>159</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
         <v>41</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>121</v>
+        <v>160</v>
       </c>
       <c r="C41" t="s" s="2">
-        <v>122</v>
-      </c>
-      <c r="D41" s="2"/>
+        <v>161</v>
+      </c>
+      <c r="D41" t="s" s="2">
+        <v>162</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>123</v>
+        <v>163</v>
       </c>
       <c r="C42" t="s" s="2">
-        <v>124</v>
-      </c>
-      <c r="D42" s="2"/>
+        <v>164</v>
+      </c>
+      <c r="D42" t="s" s="2">
+        <v>165</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>125</v>
+        <v>166</v>
       </c>
       <c r="C43" t="s" s="2">
-        <v>126</v>
-      </c>
-      <c r="D43" s="2"/>
+        <v>167</v>
+      </c>
+      <c r="D43" t="s" s="2">
+        <v>168</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>127</v>
+        <v>169</v>
       </c>
       <c r="C44" t="s" s="2">
-        <v>128</v>
-      </c>
-      <c r="D44" s="2"/>
+        <v>170</v>
+      </c>
+      <c r="D44" t="s" s="2">
+        <v>171</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>129</v>
+        <v>172</v>
       </c>
       <c r="C45" t="s" s="2">
-        <v>130</v>
-      </c>
-      <c r="D45" s="2"/>
+        <v>173</v>
+      </c>
+      <c r="D45" t="s" s="2">
+        <v>174</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>